<commit_message>
Add annual payout schedule to profit-share sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JapmQooZPmUN4PHxFgB9iJ
</commit_message>
<xml_diff>
--- a/CEO_Offer_Calculator.xlsx
+++ b/CEO_Offer_Calculator.xlsx
@@ -18,10 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%;(0.0%);&quot;-&quot;"/>
     <numFmt numFmtId="166" formatCode="0.00%;(0.00%);&quot;-&quot;"/>
+    <numFmt numFmtId="167" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -115,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -135,6 +136,9 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -266,6 +270,16 @@
     <comment ref="B12" authorId="0" shapeId="0">
       <text>
         <t>الباقي مؤجل 12 شهرًا</t>
+      </text>
+    </comment>
+    <comment ref="B37" authorId="0" shapeId="0">
+      <text>
+        <t>عادة 3–4 أشهر</t>
+      </text>
+    </comment>
+    <comment ref="B38" authorId="0" shapeId="0">
+      <text>
+        <t>يُصرف بشرط استمراره على رأس العمل</t>
       </text>
     </comment>
   </commentList>
@@ -848,7 +862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -856,6 +870,7 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1204,6 +1219,318 @@
       <c r="A33" s="2" t="inlineStr">
         <is>
           <t>المعادلة: تحت الحد الأدنى = 0 · من 80% إلى 100% خطي 10%→15% · من 100% إلى 120% خطي 15%→20% · بعدها 20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>جدول الصرف — الحافز سنوي ويُصرف بعد اعتماد القوائم المراجعة</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>السنة المالية</t>
+        </is>
+      </c>
+      <c r="B36" s="15" t="n">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>أشهر بعد نهاية السنة لاعتماد القوائم</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>مدة تأجيل الجزء المؤجل (شهر)</t>
+        </is>
+      </c>
+      <c r="B38" s="15" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>البند</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>المبلغ (ريال)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>نهاية السنة المالية</t>
+        </is>
+      </c>
+      <c r="B40" s="16">
+        <f>DATE(B36,12,31)</f>
+        <v/>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>صرف الدفعة الفورية</t>
+        </is>
+      </c>
+      <c r="B41" s="16">
+        <f>EOMONTH(B40,B37)</f>
+        <v/>
+      </c>
+      <c r="C41" s="9">
+        <f>B19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>صرف الجزء المؤجل</t>
+        </is>
+      </c>
+      <c r="B42" s="16">
+        <f>EOMONTH(B41,B38)</f>
+        <v/>
+      </c>
+      <c r="C42" s="9">
+        <f>B20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>مثال على عدة سنوات — كيف تتداخل الدفعات</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>السنة المالية</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>الربح المستهدف (ريال)</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>الربح الفعلي (ريال)</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>الحافز (ريال)</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>فوري (ريال)</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>مؤجل (ريال)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="17">
+        <f>$B$36+0</f>
+        <v/>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="C46" s="5" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="D46" s="9">
+        <f>IF($B$11&gt;0,MIN(MAX(0,(IF(IF(B46=0,0,C46/B46)&lt;$B$6,0,IF(IF(B46=0,0,C46/B46)&lt;=1,$B$7+($B$8-$B$7)*(IF(B46=0,0,C46/B46)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B46=0,0,C46/B46)-1)/($B$10-1)))))*C46),$B$11),MAX(0,(IF(IF(B46=0,0,C46/B46)&lt;$B$6,0,IF(IF(B46=0,0,C46/B46)&lt;=1,$B$7+($B$8-$B$7)*(IF(B46=0,0,C46/B46)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B46=0,0,C46/B46)-1)/($B$10-1)))))*C46))</f>
+        <v/>
+      </c>
+      <c r="E46" s="9">
+        <f>D46*$B$12</f>
+        <v/>
+      </c>
+      <c r="F46" s="9">
+        <f>D46-E46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="17">
+        <f>$B$36+1</f>
+        <v/>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>24000000</v>
+      </c>
+      <c r="C47" s="5" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="D47" s="9">
+        <f>IF($B$11&gt;0,MIN(MAX(0,(IF(IF(B47=0,0,C47/B47)&lt;$B$6,0,IF(IF(B47=0,0,C47/B47)&lt;=1,$B$7+($B$8-$B$7)*(IF(B47=0,0,C47/B47)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B47=0,0,C47/B47)-1)/($B$10-1)))))*C47),$B$11),MAX(0,(IF(IF(B47=0,0,C47/B47)&lt;$B$6,0,IF(IF(B47=0,0,C47/B47)&lt;=1,$B$7+($B$8-$B$7)*(IF(B47=0,0,C47/B47)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B47=0,0,C47/B47)-1)/($B$10-1)))))*C47))</f>
+        <v/>
+      </c>
+      <c r="E47" s="9">
+        <f>D47*$B$12</f>
+        <v/>
+      </c>
+      <c r="F47" s="9">
+        <f>D47-E47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="17">
+        <f>$B$36+2</f>
+        <v/>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>28000000</v>
+      </c>
+      <c r="C48" s="5" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="D48" s="9">
+        <f>IF($B$11&gt;0,MIN(MAX(0,(IF(IF(B48=0,0,C48/B48)&lt;$B$6,0,IF(IF(B48=0,0,C48/B48)&lt;=1,$B$7+($B$8-$B$7)*(IF(B48=0,0,C48/B48)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B48=0,0,C48/B48)-1)/($B$10-1)))))*C48),$B$11),MAX(0,(IF(IF(B48=0,0,C48/B48)&lt;$B$6,0,IF(IF(B48=0,0,C48/B48)&lt;=1,$B$7+($B$8-$B$7)*(IF(B48=0,0,C48/B48)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B48=0,0,C48/B48)-1)/($B$10-1)))))*C48))</f>
+        <v/>
+      </c>
+      <c r="E48" s="9">
+        <f>D48*$B$12</f>
+        <v/>
+      </c>
+      <c r="F48" s="9">
+        <f>D48-E48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>سنة الاستلام</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>من فوري السنة السابقة</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>من مؤجل ما قبلها</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>إجمالي ما يستلمه</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="17">
+        <f>$B$36+1</f>
+        <v/>
+      </c>
+      <c r="B51" s="9">
+        <f>SUMIF($A$46:$A$48,A51-1,$E$46:$E$48)</f>
+        <v/>
+      </c>
+      <c r="C51" s="9">
+        <f>SUMIF($A$46:$A$48,A51-2,$F$46:$F$48)</f>
+        <v/>
+      </c>
+      <c r="D51" s="11">
+        <f>B51+C51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="17">
+        <f>$B$36+2</f>
+        <v/>
+      </c>
+      <c r="B52" s="9">
+        <f>SUMIF($A$46:$A$48,A52-1,$E$46:$E$48)</f>
+        <v/>
+      </c>
+      <c r="C52" s="9">
+        <f>SUMIF($A$46:$A$48,A52-2,$F$46:$F$48)</f>
+        <v/>
+      </c>
+      <c r="D52" s="11">
+        <f>B52+C52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="17">
+        <f>$B$36+3</f>
+        <v/>
+      </c>
+      <c r="B53" s="9">
+        <f>SUMIF($A$46:$A$48,A53-1,$E$46:$E$48)</f>
+        <v/>
+      </c>
+      <c r="C53" s="9">
+        <f>SUMIF($A$46:$A$48,A53-2,$F$46:$F$48)</f>
+        <v/>
+      </c>
+      <c r="D53" s="11">
+        <f>B53+C53</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="17">
+        <f>$B$36+4</f>
+        <v/>
+      </c>
+      <c r="B54" s="9">
+        <f>SUMIF($A$46:$A$48,A54-1,$E$46:$E$48)</f>
+        <v/>
+      </c>
+      <c r="C54" s="9">
+        <f>SUMIF($A$46:$A$48,A54-2,$F$46:$F$48)</f>
+        <v/>
+      </c>
+      <c r="D54" s="11">
+        <f>B54+C54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>الفوري يُصرف في السنة التالية بعد اعتماد القوائم، والمؤجل بعدها بسنة بشرط الاستمرار. الخلايا الصفراء أرقام مثال.</t>
         </is>
       </c>
     </row>
@@ -1328,7 +1655,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>السنة 1</t>
         </is>
@@ -1350,7 +1677,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>السنة 2</t>
         </is>
@@ -1372,7 +1699,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>السنة 3</t>
         </is>
@@ -1394,7 +1721,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>السنة 4</t>
         </is>
@@ -1416,7 +1743,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>السنة 5</t>
         </is>

</xml_diff>

<commit_message>
Remove bonus deferral: profit share paid in full once a year
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JapmQooZPmUN4PHxFgB9iJ
</commit_message>
<xml_diff>
--- a/CEO_Offer_Calculator.xlsx
+++ b/CEO_Offer_Calculator.xlsx
@@ -133,11 +133,11 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -267,19 +267,9 @@
         <t>يُنصح بتحديد سقف</t>
       </text>
     </comment>
-    <comment ref="B12" authorId="0" shapeId="0">
-      <text>
-        <t>الباقي مؤجل 12 شهرًا</t>
-      </text>
-    </comment>
-    <comment ref="B37" authorId="0" shapeId="0">
+    <comment ref="B13" authorId="0" shapeId="0">
       <text>
         <t>عادة 3–4 أشهر</t>
-      </text>
-    </comment>
-    <comment ref="B38" authorId="0" shapeId="0">
-      <text>
-        <t>يُصرف بشرط استمراره على رأس العمل</t>
       </text>
     </comment>
   </commentList>
@@ -862,7 +852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -870,7 +860,6 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -970,83 +959,82 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>نسبة الدفع الفوري</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="n">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+          <t>السنة المالية</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="n">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>أشهر بعد نهاية السنة لاعتماد القوائم</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>النتيجة</t>
         </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>نسبة الإنجاز</t>
-        </is>
-      </c>
-      <c r="B15" s="12">
-        <f>IF(B4=0,0,B5/B4)</f>
-        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>نسبة الحافز المستحقة</t>
+          <t>نسبة الإنجاز</t>
         </is>
       </c>
       <c r="B16" s="13">
-        <f>IF(B15&lt;$B$6,0,IF(B15&lt;=1,$B$7+($B$8-$B$7)*(B15-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(B15-1)/($B$10-1))))</f>
+        <f>IF(B4=0,0,B5/B4)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
+          <t>نسبة الحافز المستحقة</t>
+        </is>
+      </c>
+      <c r="B17" s="14">
+        <f>IF(B16&lt;$B$6,0,IF(B16&lt;=1,$B$7+($B$8-$B$7)*(B16-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(B16-1)/($B$10-1))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
           <t>الحافز قبل السقف</t>
         </is>
       </c>
-      <c r="B17" s="9">
-        <f>MAX(0,B16*B5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>الحافز المستحق</t>
-        </is>
-      </c>
-      <c r="B18" s="11">
-        <f>IF(B11&gt;0,MIN(B17,B11),B17)</f>
+      <c r="B18" s="9">
+        <f>MAX(0,B17*B5)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>يُدفع فورًا</t>
-        </is>
-      </c>
-      <c r="B19" s="9">
-        <f>B18*B12</f>
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>الحافز المستحق (يُصرف كاملًا دفعة واحدة)</t>
+        </is>
+      </c>
+      <c r="B19" s="11">
+        <f>IF(B11&gt;0,MIN(B18,B11),B18)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>مؤجل 12 شهرًا</t>
-        </is>
-      </c>
-      <c r="B20" s="9">
-        <f>B18-B19</f>
+          <t>تاريخ الصرف</t>
+        </is>
+      </c>
+      <c r="B20" s="15">
+        <f>EOMONTH(DATE(B12,12,31),B13)</f>
         <v/>
       </c>
     </row>
@@ -1080,14 +1068,14 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="n">
+      <c r="A24" s="16" t="n">
         <v>0.7</v>
       </c>
       <c r="B24" s="9">
         <f>A24*$B$4</f>
         <v/>
       </c>
-      <c r="C24" s="13">
+      <c r="C24" s="14">
         <f>IF(A24&lt;$B$6,0,IF(A24&lt;=1,$B$7+($B$8-$B$7)*(A24-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(A24-1)/($B$10-1))))</f>
         <v/>
       </c>
@@ -1097,14 +1085,14 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="14" t="n">
+      <c r="A25" s="16" t="n">
         <v>0.8</v>
       </c>
       <c r="B25" s="9">
         <f>A25*$B$4</f>
         <v/>
       </c>
-      <c r="C25" s="13">
+      <c r="C25" s="14">
         <f>IF(A25&lt;$B$6,0,IF(A25&lt;=1,$B$7+($B$8-$B$7)*(A25-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(A25-1)/($B$10-1))))</f>
         <v/>
       </c>
@@ -1114,14 +1102,14 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="14" t="n">
+      <c r="A26" s="16" t="n">
         <v>0.9</v>
       </c>
       <c r="B26" s="9">
         <f>A26*$B$4</f>
         <v/>
       </c>
-      <c r="C26" s="13">
+      <c r="C26" s="14">
         <f>IF(A26&lt;$B$6,0,IF(A26&lt;=1,$B$7+($B$8-$B$7)*(A26-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(A26-1)/($B$10-1))))</f>
         <v/>
       </c>
@@ -1131,14 +1119,14 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="14" t="n">
+      <c r="A27" s="16" t="n">
         <v>1</v>
       </c>
       <c r="B27" s="9">
         <f>A27*$B$4</f>
         <v/>
       </c>
-      <c r="C27" s="13">
+      <c r="C27" s="14">
         <f>IF(A27&lt;$B$6,0,IF(A27&lt;=1,$B$7+($B$8-$B$7)*(A27-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(A27-1)/($B$10-1))))</f>
         <v/>
       </c>
@@ -1148,14 +1136,14 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="14" t="n">
+      <c r="A28" s="16" t="n">
         <v>1.1</v>
       </c>
       <c r="B28" s="9">
         <f>A28*$B$4</f>
         <v/>
       </c>
-      <c r="C28" s="13">
+      <c r="C28" s="14">
         <f>IF(A28&lt;$B$6,0,IF(A28&lt;=1,$B$7+($B$8-$B$7)*(A28-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(A28-1)/($B$10-1))))</f>
         <v/>
       </c>
@@ -1165,14 +1153,14 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="n">
+      <c r="A29" s="16" t="n">
         <v>1.2</v>
       </c>
       <c r="B29" s="9">
         <f>A29*$B$4</f>
         <v/>
       </c>
-      <c r="C29" s="13">
+      <c r="C29" s="14">
         <f>IF(A29&lt;$B$6,0,IF(A29&lt;=1,$B$7+($B$8-$B$7)*(A29-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(A29-1)/($B$10-1))))</f>
         <v/>
       </c>
@@ -1182,14 +1170,14 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="14" t="n">
+      <c r="A30" s="16" t="n">
         <v>1.3</v>
       </c>
       <c r="B30" s="9">
         <f>A30*$B$4</f>
         <v/>
       </c>
-      <c r="C30" s="13">
+      <c r="C30" s="14">
         <f>IF(A30&lt;$B$6,0,IF(A30&lt;=1,$B$7+($B$8-$B$7)*(A30-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(A30-1)/($B$10-1))))</f>
         <v/>
       </c>
@@ -1199,14 +1187,14 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="14" t="n">
+      <c r="A31" s="16" t="n">
         <v>1.5</v>
       </c>
       <c r="B31" s="9">
         <f>A31*$B$4</f>
         <v/>
       </c>
-      <c r="C31" s="13">
+      <c r="C31" s="14">
         <f>IF(A31&lt;$B$6,0,IF(A31&lt;=1,$B$7+($B$8-$B$7)*(A31-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(A31-1)/($B$10-1))))</f>
         <v/>
       </c>
@@ -1225,313 +1213,95 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>جدول الصرف — الحافز سنوي ويُصرف بعد اعتماد القوائم المراجعة</t>
+          <t>مثال على عدة سنوات — الحافز سنوي ويُصرف كاملًا بعد اعتماد القوائم</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>السنة المالية</t>
         </is>
       </c>
-      <c r="B36" s="15" t="n">
-        <v>2027</v>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>الربح المستهدف (ريال)</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>الربح الفعلي (ريال)</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>الحافز (ريال)</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>تاريخ الصرف</t>
+        </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>أشهر بعد نهاية السنة لاعتماد القوائم</t>
-        </is>
-      </c>
-      <c r="B37" s="15" t="n">
-        <v>4</v>
+      <c r="A37" s="17">
+        <f>$B$12+0</f>
+        <v/>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="D37" s="9">
+        <f>IF($B$11&gt;0,MIN(MAX(0,(IF(IF(B37=0,0,C37/B37)&lt;$B$6,0,IF(IF(B37=0,0,C37/B37)&lt;=1,$B$7+($B$8-$B$7)*(IF(B37=0,0,C37/B37)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B37=0,0,C37/B37)-1)/($B$10-1)))))*C37),$B$11),MAX(0,(IF(IF(B37=0,0,C37/B37)&lt;$B$6,0,IF(IF(B37=0,0,C37/B37)&lt;=1,$B$7+($B$8-$B$7)*(IF(B37=0,0,C37/B37)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B37=0,0,C37/B37)-1)/($B$10-1)))))*C37))</f>
+        <v/>
+      </c>
+      <c r="E37" s="15">
+        <f>EOMONTH(DATE(A37,12,31),$B$13)</f>
+        <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>مدة تأجيل الجزء المؤجل (شهر)</t>
-        </is>
-      </c>
-      <c r="B38" s="15" t="n">
-        <v>12</v>
+      <c r="A38" s="17">
+        <f>$B$12+1</f>
+        <v/>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>24000000</v>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="D38" s="9">
+        <f>IF($B$11&gt;0,MIN(MAX(0,(IF(IF(B38=0,0,C38/B38)&lt;$B$6,0,IF(IF(B38=0,0,C38/B38)&lt;=1,$B$7+($B$8-$B$7)*(IF(B38=0,0,C38/B38)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B38=0,0,C38/B38)-1)/($B$10-1)))))*C38),$B$11),MAX(0,(IF(IF(B38=0,0,C38/B38)&lt;$B$6,0,IF(IF(B38=0,0,C38/B38)&lt;=1,$B$7+($B$8-$B$7)*(IF(B38=0,0,C38/B38)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B38=0,0,C38/B38)-1)/($B$10-1)))))*C38))</f>
+        <v/>
+      </c>
+      <c r="E38" s="15">
+        <f>EOMONTH(DATE(A38,12,31),$B$13)</f>
+        <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t>البند</t>
-        </is>
-      </c>
-      <c r="B39" s="8" t="inlineStr">
-        <is>
-          <t>التاريخ</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>المبلغ (ريال)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>نهاية السنة المالية</t>
-        </is>
-      </c>
-      <c r="B40" s="16">
-        <f>DATE(B36,12,31)</f>
-        <v/>
-      </c>
-      <c r="C40" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>صرف الدفعة الفورية</t>
-        </is>
-      </c>
-      <c r="B41" s="16">
-        <f>EOMONTH(B40,B37)</f>
-        <v/>
-      </c>
-      <c r="C41" s="9">
-        <f>B19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>صرف الجزء المؤجل</t>
-        </is>
-      </c>
-      <c r="B42" s="16">
-        <f>EOMONTH(B41,B38)</f>
-        <v/>
-      </c>
-      <c r="C42" s="9">
-        <f>B20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>مثال على عدة سنوات — كيف تتداخل الدفعات</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
-        <is>
-          <t>السنة المالية</t>
-        </is>
-      </c>
-      <c r="B45" s="8" t="inlineStr">
-        <is>
-          <t>الربح المستهدف (ريال)</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>الربح الفعلي (ريال)</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>الحافز (ريال)</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>فوري (ريال)</t>
-        </is>
-      </c>
-      <c r="F45" s="8" t="inlineStr">
-        <is>
-          <t>مؤجل (ريال)</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="17">
-        <f>$B$36+0</f>
-        <v/>
-      </c>
-      <c r="B46" s="5" t="n">
-        <v>20000000</v>
-      </c>
-      <c r="C46" s="5" t="n">
-        <v>22000000</v>
-      </c>
-      <c r="D46" s="9">
-        <f>IF($B$11&gt;0,MIN(MAX(0,(IF(IF(B46=0,0,C46/B46)&lt;$B$6,0,IF(IF(B46=0,0,C46/B46)&lt;=1,$B$7+($B$8-$B$7)*(IF(B46=0,0,C46/B46)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B46=0,0,C46/B46)-1)/($B$10-1)))))*C46),$B$11),MAX(0,(IF(IF(B46=0,0,C46/B46)&lt;$B$6,0,IF(IF(B46=0,0,C46/B46)&lt;=1,$B$7+($B$8-$B$7)*(IF(B46=0,0,C46/B46)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B46=0,0,C46/B46)-1)/($B$10-1)))))*C46))</f>
-        <v/>
-      </c>
-      <c r="E46" s="9">
-        <f>D46*$B$12</f>
-        <v/>
-      </c>
-      <c r="F46" s="9">
-        <f>D46-E46</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="17">
-        <f>$B$36+1</f>
-        <v/>
-      </c>
-      <c r="B47" s="5" t="n">
-        <v>24000000</v>
-      </c>
-      <c r="C47" s="5" t="n">
-        <v>25000000</v>
-      </c>
-      <c r="D47" s="9">
-        <f>IF($B$11&gt;0,MIN(MAX(0,(IF(IF(B47=0,0,C47/B47)&lt;$B$6,0,IF(IF(B47=0,0,C47/B47)&lt;=1,$B$7+($B$8-$B$7)*(IF(B47=0,0,C47/B47)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B47=0,0,C47/B47)-1)/($B$10-1)))))*C47),$B$11),MAX(0,(IF(IF(B47=0,0,C47/B47)&lt;$B$6,0,IF(IF(B47=0,0,C47/B47)&lt;=1,$B$7+($B$8-$B$7)*(IF(B47=0,0,C47/B47)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B47=0,0,C47/B47)-1)/($B$10-1)))))*C47))</f>
-        <v/>
-      </c>
-      <c r="E47" s="9">
-        <f>D47*$B$12</f>
-        <v/>
-      </c>
-      <c r="F47" s="9">
-        <f>D47-E47</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="17">
-        <f>$B$36+2</f>
-        <v/>
-      </c>
-      <c r="B48" s="5" t="n">
+      <c r="A39" s="17">
+        <f>$B$12+2</f>
+        <v/>
+      </c>
+      <c r="B39" s="5" t="n">
         <v>28000000</v>
       </c>
-      <c r="C48" s="5" t="n">
+      <c r="C39" s="5" t="n">
         <v>30000000</v>
       </c>
-      <c r="D48" s="9">
-        <f>IF($B$11&gt;0,MIN(MAX(0,(IF(IF(B48=0,0,C48/B48)&lt;$B$6,0,IF(IF(B48=0,0,C48/B48)&lt;=1,$B$7+($B$8-$B$7)*(IF(B48=0,0,C48/B48)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B48=0,0,C48/B48)-1)/($B$10-1)))))*C48),$B$11),MAX(0,(IF(IF(B48=0,0,C48/B48)&lt;$B$6,0,IF(IF(B48=0,0,C48/B48)&lt;=1,$B$7+($B$8-$B$7)*(IF(B48=0,0,C48/B48)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B48=0,0,C48/B48)-1)/($B$10-1)))))*C48))</f>
-        <v/>
-      </c>
-      <c r="E48" s="9">
-        <f>D48*$B$12</f>
-        <v/>
-      </c>
-      <c r="F48" s="9">
-        <f>D48-E48</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
-        <is>
-          <t>سنة الاستلام</t>
-        </is>
-      </c>
-      <c r="B50" s="8" t="inlineStr">
-        <is>
-          <t>من فوري السنة السابقة</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
-        <is>
-          <t>من مؤجل ما قبلها</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>إجمالي ما يستلمه</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="17">
-        <f>$B$36+1</f>
-        <v/>
-      </c>
-      <c r="B51" s="9">
-        <f>SUMIF($A$46:$A$48,A51-1,$E$46:$E$48)</f>
-        <v/>
-      </c>
-      <c r="C51" s="9">
-        <f>SUMIF($A$46:$A$48,A51-2,$F$46:$F$48)</f>
-        <v/>
-      </c>
-      <c r="D51" s="11">
-        <f>B51+C51</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="17">
-        <f>$B$36+2</f>
-        <v/>
-      </c>
-      <c r="B52" s="9">
-        <f>SUMIF($A$46:$A$48,A52-1,$E$46:$E$48)</f>
-        <v/>
-      </c>
-      <c r="C52" s="9">
-        <f>SUMIF($A$46:$A$48,A52-2,$F$46:$F$48)</f>
-        <v/>
-      </c>
-      <c r="D52" s="11">
-        <f>B52+C52</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="17">
-        <f>$B$36+3</f>
-        <v/>
-      </c>
-      <c r="B53" s="9">
-        <f>SUMIF($A$46:$A$48,A53-1,$E$46:$E$48)</f>
-        <v/>
-      </c>
-      <c r="C53" s="9">
-        <f>SUMIF($A$46:$A$48,A53-2,$F$46:$F$48)</f>
-        <v/>
-      </c>
-      <c r="D53" s="11">
-        <f>B53+C53</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="17">
-        <f>$B$36+4</f>
-        <v/>
-      </c>
-      <c r="B54" s="9">
-        <f>SUMIF($A$46:$A$48,A54-1,$E$46:$E$48)</f>
-        <v/>
-      </c>
-      <c r="C54" s="9">
-        <f>SUMIF($A$46:$A$48,A54-2,$F$46:$F$48)</f>
-        <v/>
-      </c>
-      <c r="D54" s="11">
-        <f>B54+C54</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>الفوري يُصرف في السنة التالية بعد اعتماد القوائم، والمؤجل بعدها بسنة بشرط الاستمرار. الخلايا الصفراء أرقام مثال.</t>
-        </is>
+      <c r="D39" s="9">
+        <f>IF($B$11&gt;0,MIN(MAX(0,(IF(IF(B39=0,0,C39/B39)&lt;$B$6,0,IF(IF(B39=0,0,C39/B39)&lt;=1,$B$7+($B$8-$B$7)*(IF(B39=0,0,C39/B39)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B39=0,0,C39/B39)-1)/($B$10-1)))))*C39),$B$11),MAX(0,(IF(IF(B39=0,0,C39/B39)&lt;$B$6,0,IF(IF(B39=0,0,C39/B39)&lt;=1,$B$7+($B$8-$B$7)*(IF(B39=0,0,C39/B39)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B39=0,0,C39/B39)-1)/($B$10-1)))))*C39))</f>
+        <v/>
+      </c>
+      <c r="E39" s="15">
+        <f>EOMONTH(DATE(A39,12,31),$B$13)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -1663,7 +1433,7 @@
       <c r="B12" s="5" t="n">
         <v>60000000</v>
       </c>
-      <c r="C12" s="13">
+      <c r="C12" s="14">
         <f>IF(B12&lt;$B$4,0,MIN($B$6,$B$5+($B$6-$B$5)*(B12-$B$4)/($B$7-$B$4)))</f>
         <v/>
       </c>
@@ -1685,7 +1455,7 @@
       <c r="B13" s="5" t="n">
         <v>100000000</v>
       </c>
-      <c r="C13" s="13">
+      <c r="C13" s="14">
         <f>IF(B13&lt;$B$4,0,MIN($B$6,$B$5+($B$6-$B$5)*(B13-$B$4)/($B$7-$B$4)))</f>
         <v/>
       </c>
@@ -1707,7 +1477,7 @@
       <c r="B14" s="5" t="n">
         <v>150000000</v>
       </c>
-      <c r="C14" s="13">
+      <c r="C14" s="14">
         <f>IF(B14&lt;$B$4,0,MIN($B$6,$B$5+($B$6-$B$5)*(B14-$B$4)/($B$7-$B$4)))</f>
         <v/>
       </c>
@@ -1729,7 +1499,7 @@
       <c r="B15" s="5" t="n">
         <v>200000000</v>
       </c>
-      <c r="C15" s="13">
+      <c r="C15" s="14">
         <f>IF(B15&lt;$B$4,0,MIN($B$6,$B$5+($B$6-$B$5)*(B15-$B$4)/($B$7-$B$4)))</f>
         <v/>
       </c>
@@ -1751,7 +1521,7 @@
       <c r="B16" s="5" t="n">
         <v>300000000</v>
       </c>
-      <c r="C16" s="13">
+      <c r="C16" s="14">
         <f>IF(B16&lt;$B$4,0,MIN($B$6,$B$5+($B$6-$B$5)*(B16-$B$4)/($B$7-$B$4)))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Profit share: switch to fixed net-profit thresholds with a rate per tier
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JapmQooZPmUN4PHxFgB9iJ
</commit_message>
<xml_diff>
--- a/CEO_Offer_Calculator.xlsx
+++ b/CEO_Offer_Calculator.xlsx
@@ -116,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -133,13 +133,11 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -252,22 +250,12 @@
     <author>Claude</author>
   </authors>
   <commentList>
-    <comment ref="B4" authorId="0" shapeId="0">
-      <text>
-        <t>مثال — يعتمده مجلس الإدارة مع الموازنة</t>
-      </text>
-    </comment>
-    <comment ref="B5" authorId="0" shapeId="0">
+    <comment ref="B11" authorId="0" shapeId="0">
       <text>
         <t>من القوائم المراجعة، بعد الزكاة، بدون أرباح إعادة تقييم غير محققة</t>
       </text>
     </comment>
-    <comment ref="B11" authorId="0" shapeId="0">
-      <text>
-        <t>يُنصح بتحديد سقف</t>
-      </text>
-    </comment>
-    <comment ref="B13" authorId="0" shapeId="0">
+    <comment ref="B14" authorId="0" shapeId="0">
       <text>
         <t>عادة 3–4 أشهر</t>
       </text>
@@ -852,7 +840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -865,442 +853,286 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>الخيار أ — حافز من صافي الأرباح (15%–20%)</t>
+          <t>الخيار أ — حافز من صافي الأرباح حسب الرقم المحقق</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>لو وصل صافي الربح إلى رقم الشريحة يأخذ نسبتها من كامل صافي الربح</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
+          <t>الشرائح (عدّل الأرقام والنسب)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>الشريحة</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>إذا وصل صافي الربح إلى (ريال)</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>يأخذ نسبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>الشريحة 1</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>الشريحة 2</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>الشريحة 3</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>أقل من رقم الشريحة 1 = لا يوجد حافز</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
           <t>المدخلات</t>
         </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>صافي الربح المستهدف (ريال)</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="n">
-        <v>20000000</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>صافي الربح الفعلي (ريال)</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>22000000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>الحد الأدنى للإنجاز (لا حافز تحته)</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>النسبة عند الحد الأدنى</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>النسبة عند تحقيق الهدف 100%</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>النسبة القصوى</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>الإنجاز الذي تُبلغ عنده النسبة القصوى</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n">
-        <v>1.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>سقف الحافز السنوي (ريال، 0 = بدون سقف)</t>
+          <t>صافي الربح الفعلي (ريال)</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>0</v>
+        <v>22000000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>السنة المالية</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="n">
-        <v>2027</v>
+          <t>سقف الحافز السنوي (ريال، 0 = بدون سقف)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
+          <t>السنة المالية</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="n">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
           <t>أشهر بعد نهاية السنة لاعتماد القوائم</t>
         </is>
       </c>
-      <c r="B13" s="12" t="n">
+      <c r="B14" s="13" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>النتيجة</t>
         </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>نسبة الإنجاز</t>
-        </is>
-      </c>
-      <c r="B16" s="13">
-        <f>IF(B4=0,0,B5/B4)</f>
-        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>نسبة الحافز المستحقة</t>
+          <t>النسبة المستحقة</t>
         </is>
       </c>
       <c r="B17" s="14">
-        <f>IF(B16&lt;$B$6,0,IF(B16&lt;=1,$B$7+($B$8-$B$7)*(B16-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(B16-1)/($B$10-1))))</f>
+        <f>IF(B11&lt;$B$5,0,IF(B11&lt;$B$6,$C$5,IF(B11&lt;$B$7,$C$6,$C$7)))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>الحافز قبل السقف</t>
-        </is>
-      </c>
-      <c r="B18" s="9">
-        <f>MAX(0,B17*B5)</f>
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>الحافز المستحق (يُصرف كاملًا دفعة واحدة)</t>
+        </is>
+      </c>
+      <c r="B18" s="11">
+        <f>IF($B$12&gt;0,MIN(B17*B11,$B$12),B17*B11)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>الحافز المستحق (يُصرف كاملًا دفعة واحدة)</t>
-        </is>
-      </c>
-      <c r="B19" s="11">
-        <f>IF(B11&gt;0,MIN(B18,B11),B18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>تاريخ الصرف</t>
         </is>
       </c>
-      <c r="B20" s="15">
-        <f>EOMONTH(DATE(B12,12,31),B13)</f>
-        <v/>
+      <c r="B19" s="15">
+        <f>EOMONTH(DATE(B13,12,31),B14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>جدول سيناريوهات</t>
+        </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>جدول سيناريوهات (على نفس المستهدف)</t>
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>صافي الربح (ريال)</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>النسبة</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>الحافز (ريال)</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>نسبة الإنجاز</t>
-        </is>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>صافي الربح (ريال)</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>نسبة الحافز</t>
-        </is>
-      </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>الحافز (ريال)</t>
-        </is>
+      <c r="A23" s="5" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="B23" s="14">
+        <f>IF(A23&lt;$B$5,0,IF(A23&lt;$B$6,$C$5,IF(A23&lt;$B$7,$C$6,$C$7)))</f>
+        <v/>
+      </c>
+      <c r="C23" s="9">
+        <f>IF($B$12&gt;0,MIN(B23*A23,$B$12),B23*A23)</f>
+        <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="B24" s="9">
-        <f>A24*$B$4</f>
-        <v/>
-      </c>
-      <c r="C24" s="14">
-        <f>IF(A24&lt;$B$6,0,IF(A24&lt;=1,$B$7+($B$8-$B$7)*(A24-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(A24-1)/($B$10-1))))</f>
-        <v/>
-      </c>
-      <c r="D24" s="9">
-        <f>IF($B$11&gt;0,MIN(C24*B24,$B$11),MAX(0,C24*B24))</f>
+      <c r="A24" s="5" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="B24" s="14">
+        <f>IF(A24&lt;$B$5,0,IF(A24&lt;$B$6,$C$5,IF(A24&lt;$B$7,$C$6,$C$7)))</f>
+        <v/>
+      </c>
+      <c r="C24" s="9">
+        <f>IF($B$12&gt;0,MIN(B24*A24,$B$12),B24*A24)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="B25" s="9">
-        <f>A25*$B$4</f>
-        <v/>
-      </c>
-      <c r="C25" s="14">
-        <f>IF(A25&lt;$B$6,0,IF(A25&lt;=1,$B$7+($B$8-$B$7)*(A25-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(A25-1)/($B$10-1))))</f>
-        <v/>
-      </c>
-      <c r="D25" s="9">
-        <f>IF($B$11&gt;0,MIN(C25*B25,$B$11),MAX(0,C25*B25))</f>
+      <c r="A25" s="5" t="n">
+        <v>18000000</v>
+      </c>
+      <c r="B25" s="14">
+        <f>IF(A25&lt;$B$5,0,IF(A25&lt;$B$6,$C$5,IF(A25&lt;$B$7,$C$6,$C$7)))</f>
+        <v/>
+      </c>
+      <c r="C25" s="9">
+        <f>IF($B$12&gt;0,MIN(B25*A25,$B$12),B25*A25)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="B26" s="9">
-        <f>A26*$B$4</f>
-        <v/>
-      </c>
-      <c r="C26" s="14">
-        <f>IF(A26&lt;$B$6,0,IF(A26&lt;=1,$B$7+($B$8-$B$7)*(A26-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(A26-1)/($B$10-1))))</f>
-        <v/>
-      </c>
-      <c r="D26" s="9">
-        <f>IF($B$11&gt;0,MIN(C26*B26,$B$11),MAX(0,C26*B26))</f>
+      <c r="A26" s="5" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="B26" s="14">
+        <f>IF(A26&lt;$B$5,0,IF(A26&lt;$B$6,$C$5,IF(A26&lt;$B$7,$C$6,$C$7)))</f>
+        <v/>
+      </c>
+      <c r="C26" s="9">
+        <f>IF($B$12&gt;0,MIN(B26*A26,$B$12),B26*A26)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="B27" s="9">
-        <f>A27*$B$4</f>
-        <v/>
-      </c>
-      <c r="C27" s="14">
-        <f>IF(A27&lt;$B$6,0,IF(A27&lt;=1,$B$7+($B$8-$B$7)*(A27-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(A27-1)/($B$10-1))))</f>
-        <v/>
-      </c>
-      <c r="D27" s="9">
-        <f>IF($B$11&gt;0,MIN(C27*B27,$B$11),MAX(0,C27*B27))</f>
+      <c r="A27" s="5" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="B27" s="14">
+        <f>IF(A27&lt;$B$5,0,IF(A27&lt;$B$6,$C$5,IF(A27&lt;$B$7,$C$6,$C$7)))</f>
+        <v/>
+      </c>
+      <c r="C27" s="9">
+        <f>IF($B$12&gt;0,MIN(B27*A27,$B$12),B27*A27)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="B28" s="9">
-        <f>A28*$B$4</f>
-        <v/>
-      </c>
-      <c r="C28" s="14">
-        <f>IF(A28&lt;$B$6,0,IF(A28&lt;=1,$B$7+($B$8-$B$7)*(A28-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(A28-1)/($B$10-1))))</f>
-        <v/>
-      </c>
-      <c r="D28" s="9">
-        <f>IF($B$11&gt;0,MIN(C28*B28,$B$11),MAX(0,C28*B28))</f>
+      <c r="A28" s="5" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="B28" s="14">
+        <f>IF(A28&lt;$B$5,0,IF(A28&lt;$B$6,$C$5,IF(A28&lt;$B$7,$C$6,$C$7)))</f>
+        <v/>
+      </c>
+      <c r="C28" s="9">
+        <f>IF($B$12&gt;0,MIN(B28*A28,$B$12),B28*A28)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="B29" s="9">
-        <f>A29*$B$4</f>
-        <v/>
-      </c>
-      <c r="C29" s="14">
-        <f>IF(A29&lt;$B$6,0,IF(A29&lt;=1,$B$7+($B$8-$B$7)*(A29-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(A29-1)/($B$10-1))))</f>
-        <v/>
-      </c>
-      <c r="D29" s="9">
-        <f>IF($B$11&gt;0,MIN(C29*B29,$B$11),MAX(0,C29*B29))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="16" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="B30" s="9">
-        <f>A30*$B$4</f>
-        <v/>
-      </c>
-      <c r="C30" s="14">
-        <f>IF(A30&lt;$B$6,0,IF(A30&lt;=1,$B$7+($B$8-$B$7)*(A30-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(A30-1)/($B$10-1))))</f>
-        <v/>
-      </c>
-      <c r="D30" s="9">
-        <f>IF($B$11&gt;0,MIN(C30*B30,$B$11),MAX(0,C30*B30))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="16" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="B31" s="9">
-        <f>A31*$B$4</f>
-        <v/>
-      </c>
-      <c r="C31" s="14">
-        <f>IF(A31&lt;$B$6,0,IF(A31&lt;=1,$B$7+($B$8-$B$7)*(A31-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(A31-1)/($B$10-1))))</f>
-        <v/>
-      </c>
-      <c r="D31" s="9">
-        <f>IF($B$11&gt;0,MIN(C31*B31,$B$11),MAX(0,C31*B31))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>المعادلة: تحت الحد الأدنى = 0 · من 80% إلى 100% خطي 10%→15% · من 100% إلى 120% خطي 15%→20% · بعدها 20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>مثال على عدة سنوات — الحافز سنوي ويُصرف كاملًا بعد اعتماد القوائم</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>السنة المالية</t>
-        </is>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>الربح المستهدف (ريال)</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>الربح الفعلي (ريال)</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>الحافز (ريال)</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>تاريخ الصرف</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="17">
-        <f>$B$12+0</f>
-        <v/>
-      </c>
-      <c r="B37" s="5" t="n">
-        <v>20000000</v>
-      </c>
-      <c r="C37" s="5" t="n">
-        <v>22000000</v>
-      </c>
-      <c r="D37" s="9">
-        <f>IF($B$11&gt;0,MIN(MAX(0,(IF(IF(B37=0,0,C37/B37)&lt;$B$6,0,IF(IF(B37=0,0,C37/B37)&lt;=1,$B$7+($B$8-$B$7)*(IF(B37=0,0,C37/B37)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B37=0,0,C37/B37)-1)/($B$10-1)))))*C37),$B$11),MAX(0,(IF(IF(B37=0,0,C37/B37)&lt;$B$6,0,IF(IF(B37=0,0,C37/B37)&lt;=1,$B$7+($B$8-$B$7)*(IF(B37=0,0,C37/B37)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B37=0,0,C37/B37)-1)/($B$10-1)))))*C37))</f>
-        <v/>
-      </c>
-      <c r="E37" s="15">
-        <f>EOMONTH(DATE(A37,12,31),$B$13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="17">
-        <f>$B$12+1</f>
-        <v/>
-      </c>
-      <c r="B38" s="5" t="n">
-        <v>24000000</v>
-      </c>
-      <c r="C38" s="5" t="n">
-        <v>25000000</v>
-      </c>
-      <c r="D38" s="9">
-        <f>IF($B$11&gt;0,MIN(MAX(0,(IF(IF(B38=0,0,C38/B38)&lt;$B$6,0,IF(IF(B38=0,0,C38/B38)&lt;=1,$B$7+($B$8-$B$7)*(IF(B38=0,0,C38/B38)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B38=0,0,C38/B38)-1)/($B$10-1)))))*C38),$B$11),MAX(0,(IF(IF(B38=0,0,C38/B38)&lt;$B$6,0,IF(IF(B38=0,0,C38/B38)&lt;=1,$B$7+($B$8-$B$7)*(IF(B38=0,0,C38/B38)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B38=0,0,C38/B38)-1)/($B$10-1)))))*C38))</f>
-        <v/>
-      </c>
-      <c r="E38" s="15">
-        <f>EOMONTH(DATE(A38,12,31),$B$13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="17">
-        <f>$B$12+2</f>
-        <v/>
-      </c>
-      <c r="B39" s="5" t="n">
-        <v>28000000</v>
-      </c>
-      <c r="C39" s="5" t="n">
+      <c r="A29" s="5" t="n">
         <v>30000000</v>
       </c>
-      <c r="D39" s="9">
-        <f>IF($B$11&gt;0,MIN(MAX(0,(IF(IF(B39=0,0,C39/B39)&lt;$B$6,0,IF(IF(B39=0,0,C39/B39)&lt;=1,$B$7+($B$8-$B$7)*(IF(B39=0,0,C39/B39)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B39=0,0,C39/B39)-1)/($B$10-1)))))*C39),$B$11),MAX(0,(IF(IF(B39=0,0,C39/B39)&lt;$B$6,0,IF(IF(B39=0,0,C39/B39)&lt;=1,$B$7+($B$8-$B$7)*(IF(B39=0,0,C39/B39)-$B$6)/(1-$B$6),MIN($B$9,$B$8+($B$9-$B$8)*(IF(B39=0,0,C39/B39)-1)/($B$10-1)))))*C39))</f>
-        <v/>
-      </c>
-      <c r="E39" s="15">
-        <f>EOMONTH(DATE(A39,12,31),$B$13)</f>
+      <c r="B29" s="14">
+        <f>IF(A29&lt;$B$5,0,IF(A29&lt;$B$6,$C$5,IF(A29&lt;$B$7,$C$6,$C$7)))</f>
+        <v/>
+      </c>
+      <c r="C29" s="9">
+        <f>IF($B$12&gt;0,MIN(B29*A29,$B$12),B29*A29)</f>
         <v/>
       </c>
     </row>
@@ -1425,7 +1257,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>السنة 1</t>
         </is>
@@ -1433,7 +1265,7 @@
       <c r="B12" s="5" t="n">
         <v>60000000</v>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="16">
         <f>IF(B12&lt;$B$4,0,MIN($B$6,$B$5+($B$6-$B$5)*(B12-$B$4)/($B$7-$B$4)))</f>
         <v/>
       </c>
@@ -1447,7 +1279,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>السنة 2</t>
         </is>
@@ -1455,7 +1287,7 @@
       <c r="B13" s="5" t="n">
         <v>100000000</v>
       </c>
-      <c r="C13" s="14">
+      <c r="C13" s="16">
         <f>IF(B13&lt;$B$4,0,MIN($B$6,$B$5+($B$6-$B$5)*(B13-$B$4)/($B$7-$B$4)))</f>
         <v/>
       </c>
@@ -1469,7 +1301,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>السنة 3</t>
         </is>
@@ -1477,7 +1309,7 @@
       <c r="B14" s="5" t="n">
         <v>150000000</v>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="16">
         <f>IF(B14&lt;$B$4,0,MIN($B$6,$B$5+($B$6-$B$5)*(B14-$B$4)/($B$7-$B$4)))</f>
         <v/>
       </c>
@@ -1491,7 +1323,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>السنة 4</t>
         </is>
@@ -1499,7 +1331,7 @@
       <c r="B15" s="5" t="n">
         <v>200000000</v>
       </c>
-      <c r="C15" s="14">
+      <c r="C15" s="16">
         <f>IF(B15&lt;$B$4,0,MIN($B$6,$B$5+($B$6-$B$5)*(B15-$B$4)/($B$7-$B$4)))</f>
         <v/>
       </c>
@@ -1513,7 +1345,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>السنة 5</t>
         </is>
@@ -1521,7 +1353,7 @@
       <c r="B16" s="5" t="n">
         <v>300000000</v>
       </c>
-      <c r="C16" s="14">
+      <c r="C16" s="16">
         <f>IF(B16&lt;$B$4,0,MIN($B$6,$B$5+($B$6-$B$5)*(B16-$B$4)/($B$7-$B$4)))</f>
         <v/>
       </c>

</xml_diff>